<commit_message>
feat: update HTML report structure and midterm presentation slides data
</commit_message>
<xml_diff>
--- a/Formative Study/Recruitment/Ques Output.xlsx
+++ b/Formative Study/Recruitment/Ques Output.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="29120" windowHeight="12900" activeTab="1"/>
+    <workbookView windowWidth="29120" windowHeight="12900" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="初版" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="715" uniqueCount="300">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="715" uniqueCount="303">
   <si>
     <t>是否访谈</t>
   </si>
@@ -77,6 +77,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t>9</t>
     </r>
     <r>
@@ -133,6 +139,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t>12</t>
     </r>
     <r>
@@ -654,6 +666,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t>489</t>
     </r>
     <r>
@@ -860,6 +878,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
       <t>演示幻灯片（</t>
     </r>
     <r>
@@ -985,6 +1009,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve">AI </t>
     </r>
     <r>
@@ -999,6 +1029,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve">AI </t>
     </r>
     <r>
@@ -1013,6 +1049,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
       <t>常用的人与</t>
     </r>
     <r>
@@ -1036,6 +1078,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve">AI </t>
     </r>
     <r>
@@ -1050,6 +1098,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
       <t>理想的</t>
     </r>
     <r>
@@ -1076,6 +1130,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
       <t>演示幻灯片（</t>
     </r>
     <r>
@@ -1136,6 +1196,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
       <t>课程</t>
     </r>
     <r>
@@ -1159,6 +1225,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
       <t>对话大模型（</t>
     </r>
     <r>
@@ -1329,6 +1401,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve">gpt </t>
     </r>
     <r>
@@ -1388,6 +1466,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
       <t>信息图</t>
     </r>
     <r>
@@ -1467,6 +1551,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
       <t>课程</t>
     </r>
     <r>
@@ -1527,6 +1617,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
       <t>对话大模型（</t>
     </r>
     <r>
@@ -1587,6 +1683,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve">AI </t>
     </r>
     <r>
@@ -1642,6 +1744,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
       <t>演示幻灯片（</t>
     </r>
     <r>
@@ -1684,6 +1792,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
       <t>课程</t>
     </r>
     <r>
@@ -1744,6 +1858,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
       <t>对话大模型（</t>
     </r>
     <r>
@@ -1877,6 +1997,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
       <t>脑子里有想法，但很难稳定地传达给</t>
     </r>
     <r>
@@ -1937,10 +2063,218 @@
     </r>
   </si>
   <si>
+    <r>
+      <t>可以给出我框架</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
+      <t>我可以进行</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FFC00000"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
+      <t>复用</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
+      <t>但是设计过程还是要以我为主</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve"> ai</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
+      <t>起到</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
+      <t>开始时候框架定调、进行过程中润色、结束设计后评估</t>
+    </r>
+  </si>
+  <si>
     <t>gemini</t>
   </si>
   <si>
-    <r>
+    <t>周三晚上8:00</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
+      <t>其他〖</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t>ui</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
+      <t>〗</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
+      <t>脑子里有想法，但很难稳定地传达给</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve"> AI
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
+      <t>为了接近预期，只能反复改</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve"> prompt</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
+      <t>，反复试错</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">
+AI </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
+      <t>偶尔能做出不错的结果，但过程不可控、结果不稳定</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>给一个框架后，我们再一起修改，</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FFC00000"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
+      <t>先定步骤</t>
+    </r>
+  </si>
+  <si>
+    <t>codex</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
       <t>演示幻灯片（</t>
     </r>
     <r>
@@ -2001,6 +2335,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
       <t>客户提案</t>
     </r>
     <r>
@@ -2024,6 +2364,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
       <t>对话大模型（</t>
     </r>
     <r>
@@ -2120,6 +2466,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
       <t>海报</t>
     </r>
     <r>
@@ -2199,6 +2551,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
       <t>课程</t>
     </r>
     <r>
@@ -2296,6 +2654,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
       <t>对话大模型（</t>
     </r>
     <r>
@@ -2504,16 +2868,105 @@
   </si>
   <si>
     <r>
-      <t>脑子里有想法，但很难稳定地传达给</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve"> AI
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
+      <t>制作一个简单的营销活动</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t>banner</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
+      <t>或海报；或者，用类似</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t>trae</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
+      <t>的工具转换</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t>ui</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
+      <t>页面生成可交互的前端代码</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
+      <t>演示幻灯片（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t>PPT</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
+      <t>）</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">
 </t>
     </r>
     <r>
@@ -2523,25 +2976,140 @@
         <rFont val="宋体-简"/>
         <charset val="134"/>
       </rPr>
-      <t>为了接近预期，只能反复改</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve"> prompt</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="宋体-简"/>
-        <charset val="134"/>
-      </rPr>
-      <t>，反复试错</t>
+      <t>信息图</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
+      <t>社媒视觉物料（如小红书</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve"> / </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
+      <t>公众号封面）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
+      <t>课程</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve"> / </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
+      <t>学术汇报
+工作汇报</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve"> / </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
+      <t>内部沟通
+数据分析</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve"> / </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
+      <t>报告输出</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
+      <t>对话大模型（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">ChatGPT / Claude / Gemini / </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
+      <t>豆包等）</t>
     </r>
     <r>
       <rPr>
@@ -2560,89 +3128,73 @@
         <rFont val="宋体-简"/>
         <charset val="134"/>
       </rPr>
+      <t>辅助设计工具（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">Figma Make / Canva AI </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
+      <t>等）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
+      <t>为了接近预期，只能反复改</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve"> prompt</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
+      <t>，反复试错</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">
+AI </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
       <t>偶尔能做出不错的结果，但过程不可控、结果不稳定</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>制作一个简单的营销活动</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <charset val="134"/>
-      </rPr>
-      <t>banner</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="宋体-简"/>
-        <charset val="134"/>
-      </rPr>
-      <t>或海报；或者，用类似</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <charset val="134"/>
-      </rPr>
-      <t>trae</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="宋体-简"/>
-        <charset val="134"/>
-      </rPr>
-      <t>的工具转换</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <charset val="134"/>
-      </rPr>
-      <t>ui</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="宋体-简"/>
-        <charset val="134"/>
-      </rPr>
-      <t>页面生成可交互的前端代码</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>演示幻灯片（</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <charset val="134"/>
-      </rPr>
-      <t>PPT</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="宋体-简"/>
-        <charset val="134"/>
-      </rPr>
-      <t>）</t>
     </r>
     <r>
       <rPr>
@@ -2661,7 +3213,36 @@
         <rFont val="宋体-简"/>
         <charset val="134"/>
       </rPr>
-      <t>信息图</t>
+      <t>好不容易摸索出有效做法，下次换个任务又很难继续用</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
+      <t>演示幻灯片（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t>PPT</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
+      <t>）</t>
     </r>
     <r>
       <rPr>
@@ -2680,7 +3261,36 @@
         <rFont val="宋体-简"/>
         <charset val="134"/>
       </rPr>
-      <t>社媒视觉物料（如小红书</t>
+      <t>其他〖</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t>figma .md</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
+      <t>〗</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
+      <t>课程</t>
     </r>
     <r>
       <rPr>
@@ -2698,170 +3308,7 @@
         <rFont val="宋体-简"/>
         <charset val="134"/>
       </rPr>
-      <t>公众号封面）</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>课程</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve"> / </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="宋体-简"/>
-        <charset val="134"/>
-      </rPr>
-      <t>学术汇报
-工作汇报</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve"> / </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="宋体-简"/>
-        <charset val="134"/>
-      </rPr>
-      <t>内部沟通
-数据分析</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve"> / </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="宋体-简"/>
-        <charset val="134"/>
-      </rPr>
-      <t>报告输出</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>对话大模型（</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve">ChatGPT / Claude / Gemini / </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="宋体-简"/>
-        <charset val="134"/>
-      </rPr>
-      <t>豆包等）</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve">
-AI </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="宋体-简"/>
-        <charset val="134"/>
-      </rPr>
-      <t>辅助设计工具（</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve">Figma Make / Canva AI </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="宋体-简"/>
-        <charset val="134"/>
-      </rPr>
-      <t>等）</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>为了接近预期，只能反复改</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve"> prompt</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="宋体-简"/>
-        <charset val="134"/>
-      </rPr>
-      <t>，反复试错</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve">
-AI </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="宋体-简"/>
-        <charset val="134"/>
-      </rPr>
-      <t>偶尔能做出不错的结果，但过程不可控、结果不稳定</t>
+      <t>学术汇报</t>
     </r>
     <r>
       <rPr>
@@ -2880,56 +3327,25 @@
         <rFont val="宋体-简"/>
         <charset val="134"/>
       </rPr>
-      <t>好不容易摸索出有效做法，下次换个任务又很难继续用</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>其他〖</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <charset val="134"/>
-      </rPr>
-      <t>ui</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="宋体-简"/>
-        <charset val="134"/>
-      </rPr>
-      <t>〗</t>
-    </r>
-  </si>
-  <si>
-    <t>codex</t>
-  </si>
-  <si>
-    <r>
-      <t>演示幻灯片（</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <charset val="134"/>
-      </rPr>
-      <t>PPT</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="宋体-简"/>
-        <charset val="134"/>
-      </rPr>
-      <t>）</t>
+      <t>工作汇报</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve"> / </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
+      <t>内部沟通</t>
     </r>
     <r>
       <rPr>
@@ -2948,30 +3364,7 @@
         <rFont val="宋体-简"/>
         <charset val="134"/>
       </rPr>
-      <t>其他〖</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <charset val="134"/>
-      </rPr>
-      <t>figma .md</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="宋体-简"/>
-        <charset val="134"/>
-      </rPr>
-      <t>〗</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>课程</t>
+      <t>数据分析</t>
     </r>
     <r>
       <rPr>
@@ -2989,85 +3382,17 @@
         <rFont val="宋体-简"/>
         <charset val="134"/>
       </rPr>
-      <t>学术汇报</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="宋体-简"/>
-        <charset val="134"/>
-      </rPr>
-      <t>工作汇报</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve"> / </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="宋体-简"/>
-        <charset val="134"/>
-      </rPr>
-      <t>内部沟通</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="宋体-简"/>
-        <charset val="134"/>
-      </rPr>
-      <t>数据分析</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve"> / </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="宋体-简"/>
-        <charset val="134"/>
-      </rPr>
       <t>报告输出</t>
     </r>
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
       <t>对话大模型（</t>
     </r>
     <r>
@@ -3165,6 +3490,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
       <t>脑子里有想法，但很难稳定地传达给</t>
     </r>
     <r>
@@ -3220,7 +3551,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="28">
+  <fonts count="29">
     <font>
       <sz val="10"/>
       <color theme="1"/>
@@ -3418,6 +3749,12 @@
       <name val="等线"/>
       <charset val="0"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFC00000"/>
+      <name val="宋体-简"/>
+      <charset val="134"/>
     </font>
   </fonts>
   <fills count="42">
@@ -3791,7 +4128,7 @@
     </border>
   </borders>
   <cellStyleXfs count="55">
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="43" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -3945,7 +4282,7 @@
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -3998,13 +4335,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="49" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49" applyAlignment="1">
@@ -4671,7 +5005,7 @@
       </c>
     </row>
     <row r="3" ht="84" customHeight="1" spans="1:22">
-      <c r="A3" s="27" t="s">
+      <c r="A3" s="26" t="s">
         <v>22</v>
       </c>
       <c r="B3" s="5" t="s">
@@ -4739,7 +5073,7 @@
       </c>
     </row>
     <row r="4" ht="58" spans="1:22">
-      <c r="A4" s="28" t="s">
+      <c r="A4" s="27" t="s">
         <v>44</v>
       </c>
       <c r="B4" s="5" t="s">
@@ -4807,7 +5141,7 @@
       </c>
     </row>
     <row r="5" ht="29" spans="1:22">
-      <c r="A5" s="28" t="s">
+      <c r="A5" s="27" t="s">
         <v>44</v>
       </c>
       <c r="B5" s="5" t="s">
@@ -4861,7 +5195,7 @@
       <c r="R5" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="S5" s="26" t="s">
+      <c r="S5" s="25" t="s">
         <v>69</v>
       </c>
       <c r="T5" s="5" t="s">
@@ -4875,7 +5209,7 @@
       </c>
     </row>
     <row r="6" ht="72" spans="1:22">
-      <c r="A6" s="28" t="s">
+      <c r="A6" s="27" t="s">
         <v>44</v>
       </c>
       <c r="B6" s="5" t="s">
@@ -4943,7 +5277,7 @@
       </c>
     </row>
     <row r="7" ht="87" spans="1:22">
-      <c r="A7" s="27" t="s">
+      <c r="A7" s="26" t="s">
         <v>22</v>
       </c>
       <c r="B7" s="5" t="s">
@@ -5011,7 +5345,7 @@
       </c>
     </row>
     <row r="8" ht="72" spans="1:22">
-      <c r="A8" s="28" t="s">
+      <c r="A8" s="27" t="s">
         <v>44</v>
       </c>
       <c r="B8" s="5" t="s">
@@ -5044,7 +5378,7 @@
       <c r="K8" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="L8" s="26" t="s">
+      <c r="L8" s="25" t="s">
         <v>106</v>
       </c>
       <c r="M8" s="5" t="s">
@@ -5065,10 +5399,10 @@
       <c r="R8" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="S8" s="26" t="s">
+      <c r="S8" s="25" t="s">
         <v>111</v>
       </c>
-      <c r="T8" s="29" t="s">
+      <c r="T8" s="28" t="s">
         <v>112</v>
       </c>
       <c r="U8" s="5" t="s">
@@ -5079,7 +5413,7 @@
       </c>
     </row>
     <row r="9" ht="47" customHeight="1" spans="1:22">
-      <c r="A9" s="27" t="s">
+      <c r="A9" s="26" t="s">
         <v>114</v>
       </c>
       <c r="B9" s="5" t="s">
@@ -5147,7 +5481,7 @@
       </c>
     </row>
     <row r="10" ht="44" spans="1:22">
-      <c r="A10" s="27" t="s">
+      <c r="A10" s="26" t="s">
         <v>114</v>
       </c>
       <c r="B10" s="5" t="s">
@@ -5215,7 +5549,7 @@
       </c>
     </row>
     <row r="11" ht="58" spans="1:22">
-      <c r="A11" s="27" t="s">
+      <c r="A11" s="26" t="s">
         <v>22</v>
       </c>
       <c r="B11" s="5" t="s">
@@ -5283,7 +5617,7 @@
       </c>
     </row>
     <row r="12" ht="58" spans="1:22">
-      <c r="A12" s="27" t="s">
+      <c r="A12" s="26" t="s">
         <v>22</v>
       </c>
       <c r="B12" s="5" t="s">
@@ -5351,7 +5685,7 @@
       </c>
     </row>
     <row r="13" ht="58" spans="1:22">
-      <c r="A13" s="27" t="s">
+      <c r="A13" s="26" t="s">
         <v>22</v>
       </c>
       <c r="B13" s="5" t="s">
@@ -5405,7 +5739,7 @@
       <c r="R13" s="5" t="s">
         <v>169</v>
       </c>
-      <c r="S13" s="26" t="s">
+      <c r="S13" s="25" t="s">
         <v>170</v>
       </c>
       <c r="T13" s="5" t="s">
@@ -5419,7 +5753,7 @@
       </c>
     </row>
     <row r="14" ht="58" spans="1:22">
-      <c r="A14" s="27" t="s">
+      <c r="A14" s="26" t="s">
         <v>114</v>
       </c>
       <c r="B14" s="5" t="s">
@@ -5487,7 +5821,7 @@
       </c>
     </row>
     <row r="15" ht="58" spans="1:22">
-      <c r="A15" s="27" t="s">
+      <c r="A15" s="26" t="s">
         <v>22</v>
       </c>
       <c r="B15" s="5" t="s">
@@ -5555,7 +5889,7 @@
       </c>
     </row>
     <row r="16" ht="44" spans="1:22">
-      <c r="A16" s="28" t="s">
+      <c r="A16" s="27" t="s">
         <v>44</v>
       </c>
       <c r="B16" s="5" t="s">
@@ -5588,7 +5922,7 @@
       <c r="K16" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="L16" s="26" t="s">
+      <c r="L16" s="25" t="s">
         <v>202</v>
       </c>
       <c r="M16" s="5" t="s">
@@ -5609,7 +5943,7 @@
       <c r="R16" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="S16" s="26" t="s">
+      <c r="S16" s="25" t="s">
         <v>205</v>
       </c>
       <c r="T16" s="5" t="s">
@@ -5623,7 +5957,7 @@
       </c>
     </row>
     <row r="17" ht="51" customHeight="1" spans="1:22">
-      <c r="A17" s="28" t="s">
+      <c r="A17" s="27" t="s">
         <v>44</v>
       </c>
       <c r="B17" s="5" t="s">
@@ -5691,7 +6025,7 @@
       </c>
     </row>
     <row r="18" ht="44" spans="1:22">
-      <c r="A18" s="27" t="s">
+      <c r="A18" s="26" t="s">
         <v>22</v>
       </c>
       <c r="B18" s="5" t="s">
@@ -5798,70 +6132,70 @@
   </cols>
   <sheetData>
     <row r="1" ht="21" customHeight="1"/>
-    <row r="2" s="21" customFormat="1" ht="20" customHeight="1" spans="1:20">
-      <c r="A2" s="22" t="s">
+    <row r="2" s="20" customFormat="1" ht="20" customHeight="1" spans="1:20">
+      <c r="A2" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="23" t="s">
+      <c r="B2" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="23" t="s">
+      <c r="C2" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="23" t="s">
+      <c r="D2" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="22" t="s">
+      <c r="E2" s="21" t="s">
         <v>234</v>
       </c>
-      <c r="F2" s="22" t="s">
+      <c r="F2" s="21" t="s">
         <v>235</v>
       </c>
-      <c r="G2" s="22" t="s">
+      <c r="G2" s="21" t="s">
         <v>236</v>
       </c>
-      <c r="H2" s="22" t="s">
+      <c r="H2" s="21" t="s">
         <v>237</v>
       </c>
-      <c r="I2" s="23" t="s">
+      <c r="I2" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="J2" s="23" t="s">
+      <c r="J2" s="22" t="s">
         <v>9</v>
       </c>
-      <c r="K2" s="23" t="s">
+      <c r="K2" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="L2" s="23" t="s">
+      <c r="L2" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="M2" s="23" t="s">
+      <c r="M2" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="N2" s="23" t="s">
+      <c r="N2" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="O2" s="23" t="s">
+      <c r="O2" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="P2" s="23" t="s">
+      <c r="P2" s="22" t="s">
         <v>238</v>
       </c>
-      <c r="Q2" s="23" t="s">
+      <c r="Q2" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="R2" s="23" t="s">
+      <c r="R2" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="S2" s="23" t="s">
+      <c r="S2" s="22" t="s">
         <v>239</v>
       </c>
-      <c r="T2" s="23" t="s">
+      <c r="T2" s="22" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="3" s="1" customFormat="1" ht="72" spans="1:20">
-      <c r="A3" s="24" t="s">
+      <c r="A3" s="23" t="s">
         <v>22</v>
       </c>
       <c r="B3" s="5">
@@ -5923,7 +6257,7 @@
       </c>
     </row>
     <row r="4" s="1" customFormat="1" ht="58" spans="1:20">
-      <c r="A4" s="24" t="s">
+      <c r="A4" s="23" t="s">
         <v>22</v>
       </c>
       <c r="B4" s="5">
@@ -5985,7 +6319,7 @@
       </c>
     </row>
     <row r="5" s="1" customFormat="1" ht="58" spans="1:20">
-      <c r="A5" s="24" t="s">
+      <c r="A5" s="23" t="s">
         <v>22</v>
       </c>
       <c r="B5" s="5">
@@ -6047,7 +6381,7 @@
       </c>
     </row>
     <row r="6" s="1" customFormat="1" ht="29" spans="1:20">
-      <c r="A6" s="24" t="s">
+      <c r="A6" s="23" t="s">
         <v>22</v>
       </c>
       <c r="B6" s="5">
@@ -6109,7 +6443,7 @@
       </c>
     </row>
     <row r="7" s="1" customFormat="1" ht="44" spans="1:20">
-      <c r="A7" s="25" t="s">
+      <c r="A7" s="24" t="s">
         <v>246</v>
       </c>
       <c r="B7" s="5"/>
@@ -6170,7 +6504,7 @@
       <c r="F8" s="8"/>
     </row>
     <row r="11" s="1" customFormat="1" ht="58" spans="1:20">
-      <c r="A11" s="24" t="s">
+      <c r="A11" s="23" t="s">
         <v>22</v>
       </c>
       <c r="B11" s="5">
@@ -6230,7 +6564,7 @@
       </c>
     </row>
     <row r="12" s="1" customFormat="1" ht="44" spans="1:20">
-      <c r="A12" s="24" t="s">
+      <c r="A12" s="23" t="s">
         <v>22</v>
       </c>
       <c r="B12" s="5">
@@ -6292,7 +6626,7 @@
       </c>
     </row>
     <row r="13" s="1" customFormat="1" ht="87" spans="1:20">
-      <c r="A13" s="24" t="s">
+      <c r="A13" s="23" t="s">
         <v>22</v>
       </c>
       <c r="B13" s="5">
@@ -6354,7 +6688,7 @@
       </c>
     </row>
     <row r="14" s="1" customFormat="1" ht="58" spans="1:20">
-      <c r="A14" s="24" t="s">
+      <c r="A14" s="23" t="s">
         <v>22</v>
       </c>
       <c r="B14" s="5">
@@ -6414,7 +6748,7 @@
       </c>
     </row>
     <row r="15" s="1" customFormat="1" ht="58" spans="1:20">
-      <c r="A15" s="25" t="s">
+      <c r="A15" s="24" t="s">
         <v>246</v>
       </c>
       <c r="B15" s="5"/>
@@ -6464,7 +6798,7 @@
       <c r="R15" s="5" t="s">
         <v>169</v>
       </c>
-      <c r="S15" s="26" t="s">
+      <c r="S15" s="25" t="s">
         <v>170</v>
       </c>
       <c r="T15" s="5" t="s">
@@ -6496,7 +6830,7 @@
     <col min="6" max="6" width="7.95535714285714" style="1" customWidth="1"/>
     <col min="7" max="7" width="11.2857142857143" style="1" customWidth="1"/>
     <col min="8" max="8" width="13.0803571428571" style="1" customWidth="1"/>
-    <col min="9" max="9" width="27.4464285714286" style="1" customWidth="1"/>
+    <col min="9" max="9" width="28.7321428571429" style="1" customWidth="1"/>
     <col min="10" max="10" width="35.6607142857143" style="1" customWidth="1"/>
     <col min="11" max="11" width="22.5803571428571" style="1" customWidth="1"/>
     <col min="12" max="12" width="56.4375" style="1" customWidth="1"/>
@@ -6653,7 +6987,7 @@
       <c r="O4" s="17" t="s">
         <v>274</v>
       </c>
-      <c r="P4" s="18" t="s">
+      <c r="P4" s="16" t="s">
         <v>231</v>
       </c>
       <c r="Q4" s="16" t="s">
@@ -6703,25 +7037,25 @@
       <c r="O5" s="6" t="s">
         <v>279</v>
       </c>
-      <c r="P5" s="16" t="s">
-        <v>156</v>
-      </c>
-      <c r="Q5" s="18" t="s">
+      <c r="P5" s="18" t="s">
         <v>280</v>
+      </c>
+      <c r="Q5" s="16" t="s">
+        <v>281</v>
       </c>
     </row>
     <row r="6" s="1" customFormat="1" ht="90" customHeight="1" spans="2:17">
       <c r="B6" s="5">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>178</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>251</v>
+        <v>190</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>282</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>184</v>
+        <v>195</v>
       </c>
       <c r="F6" s="11" t="s">
         <v>105</v>
@@ -6736,63 +7070,63 @@
         <v>79</v>
       </c>
       <c r="J6" s="6" t="s">
-        <v>281</v>
-      </c>
-      <c r="K6" s="6" t="s">
-        <v>282</v>
+        <v>283</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>192</v>
       </c>
       <c r="L6" s="6" t="s">
-        <v>283</v>
+        <v>278</v>
       </c>
       <c r="M6" s="15" t="s">
         <v>37</v>
       </c>
       <c r="N6" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="O6" s="5" t="s">
-        <v>182</v>
+        <v>109</v>
+      </c>
+      <c r="O6" s="6" t="s">
+        <v>284</v>
       </c>
       <c r="P6" s="18" t="s">
-        <v>183</v>
-      </c>
-      <c r="Q6" s="18" t="s">
-        <v>280</v>
+        <v>285</v>
+      </c>
+      <c r="Q6" s="16" t="s">
+        <v>286</v>
       </c>
     </row>
     <row r="7" s="1" customFormat="1" ht="90" customHeight="1" spans="2:17">
       <c r="B7" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>91</v>
+        <v>178</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>98</v>
-      </c>
-      <c r="F7" s="10" t="s">
-        <v>30</v>
+        <v>184</v>
+      </c>
+      <c r="F7" s="11" t="s">
+        <v>105</v>
       </c>
       <c r="G7" s="5" t="s">
         <v>31</v>
       </c>
       <c r="H7" s="12" t="s">
-        <v>78</v>
-      </c>
-      <c r="I7" s="14" t="s">
-        <v>92</v>
+        <v>179</v>
+      </c>
+      <c r="I7" s="10" t="s">
+        <v>79</v>
       </c>
       <c r="J7" s="6" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="K7" s="6" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="L7" s="6" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="M7" s="15" t="s">
         <v>37</v>
@@ -6800,28 +7134,28 @@
       <c r="N7" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="O7" s="6" t="s">
-        <v>287</v>
+      <c r="O7" s="5" t="s">
+        <v>182</v>
       </c>
       <c r="P7" s="16" t="s">
-        <v>96</v>
-      </c>
-      <c r="Q7" s="20" t="s">
-        <v>288</v>
+        <v>183</v>
+      </c>
+      <c r="Q7" s="16" t="s">
+        <v>281</v>
       </c>
     </row>
     <row r="8" s="1" customFormat="1" ht="90" customHeight="1" spans="2:17">
       <c r="B8" s="5">
-        <v>6</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>244</v>
+        <v>5</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>91</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>123</v>
+        <v>98</v>
       </c>
       <c r="F8" s="10" t="s">
         <v>30</v>
@@ -6829,85 +7163,85 @@
       <c r="G8" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="H8" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="I8" s="11" t="s">
-        <v>33</v>
+      <c r="H8" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="I8" s="14" t="s">
+        <v>92</v>
       </c>
       <c r="J8" s="6" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="K8" s="6" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="L8" s="6" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="M8" s="15" t="s">
         <v>37</v>
       </c>
       <c r="N8" s="5" t="s">
-        <v>38</v>
+        <v>54</v>
       </c>
       <c r="O8" s="6" t="s">
-        <v>292</v>
+        <v>284</v>
       </c>
       <c r="P8" s="16" t="s">
-        <v>122</v>
+        <v>96</v>
       </c>
       <c r="Q8" s="18" t="s">
-        <v>57</v>
+        <v>293</v>
       </c>
     </row>
     <row r="9" s="1" customFormat="1" ht="90" customHeight="1" spans="2:17">
       <c r="B9" s="5">
-        <v>7</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>190</v>
-      </c>
-      <c r="D9" s="7" t="s">
-        <v>247</v>
+        <v>6</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>244</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>245</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>195</v>
-      </c>
-      <c r="F9" s="11" t="s">
-        <v>105</v>
+        <v>123</v>
+      </c>
+      <c r="F9" s="10" t="s">
+        <v>30</v>
       </c>
       <c r="G9" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="H9" s="12" t="s">
-        <v>179</v>
-      </c>
-      <c r="I9" s="10" t="s">
-        <v>79</v>
+      <c r="H9" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="I9" s="11" t="s">
+        <v>33</v>
       </c>
       <c r="J9" s="6" t="s">
-        <v>293</v>
-      </c>
-      <c r="K9" s="5" t="s">
-        <v>192</v>
+        <v>294</v>
+      </c>
+      <c r="K9" s="6" t="s">
+        <v>295</v>
       </c>
       <c r="L9" s="6" t="s">
-        <v>278</v>
+        <v>296</v>
       </c>
       <c r="M9" s="15" t="s">
         <v>37</v>
       </c>
       <c r="N9" s="5" t="s">
-        <v>109</v>
+        <v>38</v>
       </c>
       <c r="O9" s="6" t="s">
-        <v>287</v>
-      </c>
-      <c r="P9" s="18" t="s">
-        <v>193</v>
+        <v>297</v>
+      </c>
+      <c r="P9" s="16" t="s">
+        <v>122</v>
       </c>
       <c r="Q9" s="16" t="s">
-        <v>294</v>
+        <v>57</v>
       </c>
     </row>
     <row r="10" s="1" customFormat="1" ht="90" customHeight="1" spans="2:17">
@@ -6936,13 +7270,13 @@
         <v>79</v>
       </c>
       <c r="J10" s="6" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="K10" s="6" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="L10" s="6" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="M10" s="15" t="s">
         <v>37</v>
@@ -6951,13 +7285,13 @@
         <v>132</v>
       </c>
       <c r="O10" s="6" t="s">
-        <v>298</v>
-      </c>
-      <c r="P10" s="18" t="s">
+        <v>301</v>
+      </c>
+      <c r="P10" s="16" t="s">
         <v>145</v>
       </c>
       <c r="Q10" s="19" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
     </row>
     <row r="13" s="1" customFormat="1" spans="4:19">

</xml_diff>